<commit_message>
Refactor track_usage.py to support multiple machines and enhance data handling; update permissions in settings.local.json and add machine-specific identifier to .gitignore.
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -18,14 +18,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
@@ -40,18 +46,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3D3D3"/>
-        <bgColor rgb="00D3D3D3"/>
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFACD"/>
-        <bgColor rgb="00FFFACD"/>
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,23 +65,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,132 +455,337 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OS</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Input Tokens</t>
+          <t>Machine</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Output Tokens</t>
+          <t>Tokens</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Cache Creation Tokens</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Cache Read Tokens</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total Tokens</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>Cost ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>1502183</v>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1421466</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>85320034</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1094760399</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>1183004082</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>820.11</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2025-12-14 21:04:21</t>
-        </is>
+        <v>550358</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1.37</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>macOS</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+          <t>2025-11-17</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>32022530</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>23.3</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Combined</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>1502183</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>1421466</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>85320034</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>1094760399</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>1183004082</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>820.11</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>2025-12-14 21:04:21</t>
-        </is>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>42453788</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>26.95</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>24717634</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>18.18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>42282470</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>34.38</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>5187171</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3.69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>528925</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>24994881</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>16.64</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>6476688</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>4.35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>7476426</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>4.84</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>19992388</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>10.42</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>26491616</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>11.86</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>30829943</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>17.44</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>14917453</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>1372873</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>3436255</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>2.77</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr"/>
+      <c r="C18" s="5" t="n">
+        <v>283731399</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>185.23</v>
       </c>
     </row>
   </sheetData>
@@ -580,132 +799,157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OS</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Input Tokens</t>
+          <t>Machine</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Output Tokens</t>
+          <t>Tokens</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Cache Creation Tokens</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Cache Read Tokens</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total Tokens</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>Cost ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>1502183</v>
+          <t>2025-11-10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1421466</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>85320034</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1094760399</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>1183004082</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>820.11</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2025-12-14 21:04:21</t>
-        </is>
+        <v>550358</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1.37</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>macOS</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+          <t>2025-11-17</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>74476318</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>50.25</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Combined</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>1502183</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>1421466</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>85320034</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>1094760399</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>1183004082</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>820.11</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>2025-12-14 21:04:21</t>
-        </is>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>72187275</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>56.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>39476920</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>26.21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>93604273</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>48.36</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3436255</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>2.77</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="5" t="n">
+        <v>283731399</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>185.21</v>
       </c>
     </row>
   </sheetData>
@@ -719,132 +963,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OS</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Input Tokens</t>
+          <t>Machine</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Output Tokens</t>
+          <t>Tokens</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Cache Creation Tokens</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Cache Read Tokens</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total Tokens</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>Cost ($)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>1502183</v>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1421466</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>85320034</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1094760399</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>1183004082</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>820.11</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2025-12-14 21:04:21</t>
-        </is>
+        <v>147213951</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>107.87</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>macOS</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>136517448</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>77.34</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Combined</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>1502183</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>1421466</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>85320034</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>1094760399</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>1183004082</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>820.11</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>2025-12-14 21:04:21</t>
-        </is>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="5" t="n">
+        <v>283731399</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>185.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx to reflect recent changes in data structure and usage metrics
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -507,25 +507,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>32022530</v>
+        <v>1908261</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>23.3</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -534,52 +534,52 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>42453788</v>
+        <v>32022530</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>26.95</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24717634</v>
+        <v>638255</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>18.18</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>42282470</v>
+        <v>105685515</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>34.38</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -588,70 +588,70 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>5187171</v>
+        <v>42453788</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3.69</v>
+        <v>26.95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>528925</v>
+        <v>22622711</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.39</v>
+        <v>13.73</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>24994881</v>
+        <v>4554824</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>16.64</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6476688</v>
+        <v>264353</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4.35</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -660,34 +660,34 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7476426</v>
+        <v>24717634</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4.84</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>19992388</v>
+        <v>36196467</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.42</v>
+        <v>27.69</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -696,34 +696,34 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>26491616</v>
+        <v>42282470</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>11.86</v>
+        <v>34.38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>30829943</v>
+        <v>134304301</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>17.44</v>
+        <v>111.33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -732,60 +732,420 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>14917453</v>
+        <v>5187171</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>7.7</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1372873</v>
+        <v>61197206</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.95</v>
+        <v>48.65</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>53296925</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>31.62</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>75311927</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>58.03</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>40068985</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>528925</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>350913</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>24994881</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>16.64</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>251054</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>6476688</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>4.35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7383521</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>5.81</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7476426</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>4.84</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>19992388</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>10.42</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>84554</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>26491616</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>11.86</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>30829943</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>17.44</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>326063</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>14917453</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>12254463</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>1372873</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>7095255</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>13.63</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>14513746</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>8.859999999999999</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
         <v>3436255</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D37" s="3" t="n">
         <v>2.77</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="5" t="n">
-        <v>283731399</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>185.23</v>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="5" t="n">
+        <v>862040698</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>604.73</v>
       </c>
     </row>
   </sheetData>
@@ -799,7 +1159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -851,25 +1211,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>74476318</v>
+        <v>1908261</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>50.25</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -878,34 +1238,34 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>72187275</v>
+        <v>74476318</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>56.25</v>
+        <v>50.25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>39476920</v>
+        <v>133765658</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>26.21</v>
+        <v>71.15000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -914,42 +1274,132 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>93604273</v>
+        <v>72187275</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>48.36</v>
+        <v>56.25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>400375811</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>310.62</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>39476920</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>26.21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>7985488</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>7.13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>93604273</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>48.36</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>34274081</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>29.43</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
         <v>3436255</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D12" s="3" t="n">
         <v>2.77</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="n">
-        <v>283731399</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>185.21</v>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="5" t="n">
+        <v>862040698</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>604.7</v>
       </c>
     </row>
   </sheetData>
@@ -963,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1015,33 +1465,69 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>536049730</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>382.93</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
         <v>136517448</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D4" s="3" t="n">
         <v>77.34</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>42259569</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>36.56</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="5" t="n">
-        <v>283731399</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>185.21</v>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="5" t="n">
+        <v>862040698</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>604.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx to incorporate new data structure and metrics
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -507,97 +507,97 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-11-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1908261</v>
+        <v>49724464</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.16</v>
+        <v>39.07</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>32022530</v>
+        <v>1908261</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.3</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>638255</v>
+        <v>21866795</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.99</v>
+        <v>10.71</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>105685515</v>
+        <v>32022530</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>53.8</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>42453788</v>
+        <v>638255</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>26.95</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -606,34 +606,34 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>22622711</v>
+        <v>105685515</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>13.73</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>4554824</v>
+        <v>42453788</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2.34</v>
+        <v>26.95</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -642,34 +642,34 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>264353</v>
+        <v>22622711</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.29</v>
+        <v>13.73</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>24717634</v>
+        <v>2749441</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>18.18</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -678,34 +678,34 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>36196467</v>
+        <v>4554824</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>27.69</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>42282470</v>
+        <v>32445325</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>34.38</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -714,52 +714,52 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>134304301</v>
+        <v>264353</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>111.33</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>5187171</v>
+        <v>25621364</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3.69</v>
+        <v>16.13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>61197206</v>
+        <v>24717634</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>48.65</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -768,34 +768,34 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>53296925</v>
+        <v>36196467</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>31.62</v>
+        <v>27.69</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>75311927</v>
+        <v>42282470</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>58.03</v>
+        <v>34.38</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -804,16 +804,16 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>40068985</v>
+        <v>134304301</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>33.3</v>
+        <v>111.33</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -822,16 +822,16 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>528925</v>
+        <v>5187171</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.39</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -840,142 +840,142 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>350913</v>
+        <v>61197206</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.41</v>
+        <v>48.65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>24994881</v>
+        <v>53296925</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>16.64</v>
+        <v>31.62</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>251054</v>
+        <v>10092380</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.91</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>6476688</v>
+        <v>75311927</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>4.35</v>
+        <v>58.03</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>7383521</v>
+        <v>5756303</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>5.81</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>7476426</v>
+        <v>40068985</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>4.84</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>19992388</v>
+        <v>30795369</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>10.42</v>
+        <v>20.06</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>84554</v>
+        <v>45337137</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.35</v>
+        <v>38.62</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -984,34 +984,34 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>26491616</v>
+        <v>528925</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>11.86</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>30829943</v>
+        <v>13396201</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>17.44</v>
+        <v>13.78</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1020,132 +1020,564 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>326063</v>
+        <v>350913</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.51</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>14917453</v>
+        <v>55639860</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>7.7</v>
+        <v>44.62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>12254463</v>
+        <v>24994881</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>6.09</v>
+        <v>16.64</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1372873</v>
+        <v>251054</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.95</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>7095255</v>
+        <v>41742778</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>13.63</v>
+        <v>31.88</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14513746</v>
+        <v>6476688</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>8.859999999999999</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>7383521</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>5.81</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>125222974</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>109.87</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>7476426</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>4.84</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>129389519</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>89.77</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-12-06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>182790445</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>131.82</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>93108283</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>61.4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>19992388</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>10.42</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>84554</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>28210903</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>14.03</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>26491616</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>11.86</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>10194888</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>30829943</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>17.44</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>326063</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>74361574</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>47.89</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>14917453</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>12254463</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>127677963</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>70.15000000000001</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>1372873</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>7095255</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>13.63</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>32230252</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>18.26</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>13717170</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>7.85</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>14513746</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>8.859999999999999</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>30932694</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
         <v>3436255</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D60" s="3" t="n">
         <v>2.77</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>427250</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr"/>
-      <c r="C38" s="5" t="n">
-        <v>862040698</v>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>604.73</v>
+      <c r="B62" s="4" t="inlineStr"/>
+      <c r="C62" s="5" t="n">
+        <v>2045472030</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>1425.1</v>
       </c>
     </row>
   </sheetData>
@@ -1159,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1229,19 +1661,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>74476318</v>
+        <v>71591259</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>50.25</v>
+        <v>49.77</v>
       </c>
     </row>
     <row r="5">
@@ -1252,56 +1684,56 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>133765658</v>
+        <v>74476318</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>71.15000000000001</v>
+        <v>50.25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>72187275</v>
+        <v>133765658</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>56.25</v>
+        <v>71.15000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>400375811</v>
+        <v>60816130</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>310.62</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1310,16 +1742,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>39476920</v>
+        <v>72187275</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>26.21</v>
+        <v>56.25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1328,78 +1760,186 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7985488</v>
+        <v>400375811</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7.13</v>
+        <v>310.62</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>93604273</v>
+        <v>91981189</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>48.36</v>
+        <v>67.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>34274081</v>
+        <v>39476920</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>29.43</v>
+        <v>26.21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>7985488</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>7.13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>641290060</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>483.15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>93604273</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>48.36</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>34274081</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>29.43</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>317325444</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>181.54</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
         <v>3436255</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D17" s="3" t="n">
         <v>2.77</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>427250</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="5" t="n">
-        <v>862040698</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>604.7</v>
+      <c r="B19" s="4" t="inlineStr"/>
+      <c r="C19" s="5" t="n">
+        <v>2045472030</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>1425.08</v>
       </c>
     </row>
   </sheetData>
@@ -1413,7 +1953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1483,19 +2023,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>136517448</v>
+        <v>224388578</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>77.34</v>
+        <v>155.43</v>
       </c>
     </row>
     <row r="5">
@@ -1506,28 +2046,64 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
+        <v>136517448</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>77.34</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>42259569</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D6" s="3" t="n">
         <v>36.56</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>959042754</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>664.95</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
-      <c r="C6" s="5" t="n">
-        <v>862040698</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>604.7</v>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="5" t="n">
+        <v>2045472030</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1425.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance track_usage.py with new machine totals functionality and improve date handling; update Excel formatting and add normalization for date strings.
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machine Totals" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +502,7 @@
         <v>550358</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.37</v>
+        <v>1.3687554</v>
       </c>
     </row>
     <row r="3">
@@ -519,7 +520,7 @@
         <v>32022530</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>23.3</v>
+        <v>23.29739539999999</v>
       </c>
     </row>
     <row r="4">
@@ -537,7 +538,7 @@
         <v>42453788</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>26.95</v>
+        <v>26.95244859999999</v>
       </c>
     </row>
     <row r="5">
@@ -555,7 +556,7 @@
         <v>24717634</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>18.18</v>
+        <v>18.18267269999998</v>
       </c>
     </row>
     <row r="6">
@@ -573,7 +574,7 @@
         <v>42282470</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>34.38</v>
+        <v>34.37932540000001</v>
       </c>
     </row>
     <row r="7">
@@ -591,7 +592,7 @@
         <v>5187171</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3.69</v>
+        <v>3.687872</v>
       </c>
     </row>
     <row r="8">
@@ -609,7 +610,7 @@
         <v>528925</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.39</v>
+        <v>0.38822715</v>
       </c>
     </row>
     <row r="9">
@@ -627,7 +628,7 @@
         <v>24994881</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>16.64</v>
+        <v>16.63949649999999</v>
       </c>
     </row>
     <row r="10">
@@ -645,7 +646,7 @@
         <v>6476688</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4.35</v>
+        <v>4.3460157</v>
       </c>
     </row>
     <row r="11">
@@ -663,7 +664,7 @@
         <v>7476426</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4.84</v>
+        <v>4.83685985</v>
       </c>
     </row>
     <row r="12">
@@ -681,7 +682,7 @@
         <v>19992388</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.42</v>
+        <v>10.41620645</v>
       </c>
     </row>
     <row r="13">
@@ -699,7 +700,7 @@
         <v>26491616</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>11.86</v>
+        <v>11.8556978</v>
       </c>
     </row>
     <row r="14">
@@ -717,7 +718,7 @@
         <v>30829943</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>17.44</v>
+        <v>17.43594785000001</v>
       </c>
     </row>
     <row r="15">
@@ -735,7 +736,7 @@
         <v>14917453</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>7.7</v>
+        <v>7.702555249999997</v>
       </c>
     </row>
     <row r="16">
@@ -753,7 +754,7 @@
         <v>1372873</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.95</v>
+        <v>0.9457156999999998</v>
       </c>
     </row>
     <row r="17">
@@ -768,10 +769,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>3436255</v>
+        <v>4622790</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>2.77</v>
+        <v>3.945586</v>
       </c>
     </row>
     <row r="18">
@@ -782,10 +783,10 @@
       </c>
       <c r="B18" s="4" t="inlineStr"/>
       <c r="C18" s="5" t="n">
-        <v>283731399</v>
+        <v>284917934</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>185.23</v>
+        <v>186.38077775</v>
       </c>
     </row>
   </sheetData>
@@ -845,7 +846,7 @@
         <v>550358</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.37</v>
+        <v>1.3687554</v>
       </c>
     </row>
     <row r="3">
@@ -863,7 +864,7 @@
         <v>74476318</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>50.25</v>
+        <v>50.24984399999998</v>
       </c>
     </row>
     <row r="4">
@@ -881,7 +882,7 @@
         <v>72187275</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>56.25</v>
+        <v>56.2498701</v>
       </c>
     </row>
     <row r="5">
@@ -899,7 +900,7 @@
         <v>39476920</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>26.21</v>
+        <v>26.21059919999999</v>
       </c>
     </row>
     <row r="6">
@@ -917,7 +918,7 @@
         <v>93604273</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>48.36</v>
+        <v>48.35612305000001</v>
       </c>
     </row>
     <row r="7">
@@ -932,10 +933,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3436255</v>
+        <v>4622790</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2.77</v>
+        <v>3.945586</v>
       </c>
     </row>
     <row r="8">
@@ -946,10 +947,10 @@
       </c>
       <c r="B8" s="4" t="inlineStr"/>
       <c r="C8" s="5" t="n">
-        <v>283731399</v>
+        <v>284917934</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>185.21</v>
+        <v>186.38077775</v>
       </c>
     </row>
   </sheetData>
@@ -1009,7 +1010,7 @@
         <v>147213951</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>107.87</v>
+        <v>107.8684695</v>
       </c>
     </row>
     <row r="3">
@@ -1024,10 +1025,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>136517448</v>
+        <v>137703983</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>77.34</v>
+        <v>78.51230825</v>
       </c>
     </row>
     <row r="4">
@@ -1038,10 +1039,72 @@
       </c>
       <c r="B4" s="4" t="inlineStr"/>
       <c r="C4" s="5" t="n">
-        <v>283731399</v>
+        <v>284917934</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>185.21</v>
+        <v>186.38077775</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tokens</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cost ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>284917934</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>186.38077775</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>284917934</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>186.38077775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx to reflect changes in data structure and metrics
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -508,25 +508,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>32022530</v>
+        <v>1908261</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>23.29739539999999</v>
+        <v>1.1571819</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -535,52 +535,52 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>42453788</v>
+        <v>32022530</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>26.95244859999999</v>
+        <v>23.29739539999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>24717634</v>
+        <v>638255</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>18.18267269999998</v>
+        <v>0.9898817499999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>42282470</v>
+        <v>105685515</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>34.37932540000001</v>
+        <v>53.79845279999998</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -589,70 +589,70 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>5187171</v>
+        <v>42453788</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3.687872</v>
+        <v>26.95244859999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>528925</v>
+        <v>22622711</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.38822715</v>
+        <v>13.7266725</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>24994881</v>
+        <v>4554824</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>16.63949649999999</v>
+        <v>2.3443313</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6476688</v>
+        <v>264353</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4.3460157</v>
+        <v>0.2899901</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -661,34 +661,34 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7476426</v>
+        <v>24717634</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4.83685985</v>
+        <v>18.18267269999998</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>19992388</v>
+        <v>36196467</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.41620645</v>
+        <v>27.69193644999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -697,34 +697,34 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>26491616</v>
+        <v>42282470</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>11.8556978</v>
+        <v>34.37932540000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>30829943</v>
+        <v>134304301</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>17.43594785000001</v>
+        <v>111.3310283000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -733,60 +733,420 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>14917453</v>
+        <v>5187171</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>7.702555249999997</v>
+        <v>3.687872</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1372873</v>
+        <v>61197206</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.9457156999999998</v>
+        <v>48.65078544999998</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>53296925</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>31.6186225</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>75311927</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>58.03115755000004</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>40068985</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>33.2958544</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>528925</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.38822715</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>350913</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.4064992500000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>24994881</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>16.63949649999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>251054</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.91434825</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>6476688</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>4.3460157</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7383521</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>5.805153150000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7476426</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>4.83685985</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>19992388</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>10.41620645</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>84554</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.34924275</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>26491616</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>11.8556978</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>30829943</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>17.43594785000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>326063</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0.50919775</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>14917453</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>7.702555249999997</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>12254463</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>6.085756150000001</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>1372873</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0.9457156999999998</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>7095255</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>13.62557925</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>14513746</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>8.859738050000006</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
         <v>4622790</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D37" s="3" t="n">
         <v>3.945586</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="5" t="n">
-        <v>284917934</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>186.38077775</v>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="5" t="n">
+        <v>863227233</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>605.8621873500003</v>
       </c>
     </row>
   </sheetData>
@@ -800,7 +1160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -852,25 +1212,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>74476318</v>
+        <v>1908261</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>50.24984399999998</v>
+        <v>1.1571819</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -879,34 +1239,34 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>72187275</v>
+        <v>74476318</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>56.2498701</v>
+        <v>50.24984399999998</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>39476920</v>
+        <v>133765658</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>26.21059919999999</v>
+        <v>71.14932844999997</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -915,42 +1275,132 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>93604273</v>
+        <v>72187275</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>48.35612305000001</v>
+        <v>56.2498701</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>400375811</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>310.6193846500001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>39476920</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>26.21059919999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>7985488</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>7.126000650000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>93604273</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>48.35612305000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>34274081</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>29.42951395000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
         <v>4622790</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D12" s="3" t="n">
         <v>3.945586</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="n">
-        <v>284917934</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>186.38077775</v>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="5" t="n">
+        <v>863227233</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>605.8621873500001</v>
       </c>
     </row>
   </sheetData>
@@ -964,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1016,33 +1466,69 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>536049730</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>382.9258950000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
         <v>137703983</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D4" s="3" t="n">
         <v>78.51230825</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>42259569</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>36.55551460000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="5" t="n">
-        <v>284917934</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>186.38077775</v>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="5" t="n">
+        <v>863227233</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>605.8621873500002</v>
       </c>
     </row>
   </sheetData>
@@ -1056,7 +1542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1095,16 +1581,29 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>578309299</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>419.4814096000002</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>284917934</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>186.38077775</v>
+      <c r="B4" s="5" t="n">
+        <v>863227233</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>605.8621873500001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx to reflect recent changes in data structure and metrics
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -508,97 +508,97 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-11-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1908261</v>
+        <v>49724464</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.1571819</v>
+        <v>39.06561020000006</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>32022530</v>
+        <v>1908261</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.29739539999999</v>
+        <v>1.1571819</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>638255</v>
+        <v>21866795</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.9898817499999999</v>
+        <v>10.70585355</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>105685515</v>
+        <v>32022530</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>53.79845279999998</v>
+        <v>23.29739539999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>42453788</v>
+        <v>638255</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>26.95244859999999</v>
+        <v>0.9898817499999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -607,34 +607,34 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>22622711</v>
+        <v>105685515</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>13.7266725</v>
+        <v>53.79845279999998</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>4554824</v>
+        <v>42453788</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2.3443313</v>
+        <v>26.95244859999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -643,34 +643,34 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>264353</v>
+        <v>22622711</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.2899901</v>
+        <v>13.7266725</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>24717634</v>
+        <v>2749441</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>18.18267269999998</v>
+        <v>2.0662234</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -679,34 +679,34 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>36196467</v>
+        <v>4554824</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>27.69193644999999</v>
+        <v>2.3443313</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>42282470</v>
+        <v>32445325</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>34.37932540000001</v>
+        <v>19.70108345</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -715,52 +715,52 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>134304301</v>
+        <v>264353</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>111.3310283000001</v>
+        <v>0.2899901</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>5187171</v>
+        <v>25621364</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3.687872</v>
+        <v>16.1334694</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>61197206</v>
+        <v>24717634</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>48.65078544999998</v>
+        <v>18.18267269999998</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -769,34 +769,34 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>53296925</v>
+        <v>36196467</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>31.6186225</v>
+        <v>27.69193644999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>75311927</v>
+        <v>42282470</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>58.03115755000004</v>
+        <v>34.37932540000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -805,16 +805,16 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>40068985</v>
+        <v>134304301</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>33.2958544</v>
+        <v>111.3310283000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -823,16 +823,16 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>528925</v>
+        <v>5187171</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.38822715</v>
+        <v>3.687872</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -841,142 +841,142 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>350913</v>
+        <v>61197206</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.4064992500000001</v>
+        <v>48.65078544999998</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>24994881</v>
+        <v>53296925</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>16.63949649999999</v>
+        <v>31.6186225</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>251054</v>
+        <v>10092380</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.91434825</v>
+        <v>6.0643462</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>6476688</v>
+        <v>75311927</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>4.3460157</v>
+        <v>58.03115755000004</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>7383521</v>
+        <v>5756303</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>5.805153150000001</v>
+        <v>3.005845849999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>7476426</v>
+        <v>40068985</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>4.83685985</v>
+        <v>33.2958544</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>19992388</v>
+        <v>30795369</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>10.41620645</v>
+        <v>20.05914915000002</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>84554</v>
+        <v>45337137</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.34924275</v>
+        <v>38.62387350000002</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -985,34 +985,34 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>26491616</v>
+        <v>528925</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>11.8556978</v>
+        <v>0.38822715</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>30829943</v>
+        <v>13396201</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>17.43594785000001</v>
+        <v>13.78157245</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1021,132 +1021,564 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>326063</v>
+        <v>350913</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.50919775</v>
+        <v>0.4064992500000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>14917453</v>
+        <v>55639860</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>7.702555249999997</v>
+        <v>44.61786230000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>12254463</v>
+        <v>24994881</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>6.085756150000001</v>
+        <v>16.63949649999999</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1372873</v>
+        <v>251054</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.9457156999999998</v>
+        <v>0.91434825</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>7095255</v>
+        <v>41742778</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>13.62557925</v>
+        <v>31.88196614999998</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14513746</v>
+        <v>6476688</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>8.859738050000006</v>
+        <v>4.3460157</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>7383521</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>5.805153150000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>125222974</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>109.86724235</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>7476426</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>4.83685985</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>129389519</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>89.77331820000003</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-12-06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>182790445</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>131.8210713499999</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>93108283</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>61.40351999999999</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>19992388</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>10.41620645</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>84554</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>0.34924275</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>28210903</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>14.03307105000002</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>26491616</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>11.8556978</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>10194888</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>5.0491626</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>30829943</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>17.43594785000001</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>326063</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>0.50919775</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>74361574</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>47.88594100000003</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>14917453</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>7.702555249999997</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>12254463</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>6.085756150000001</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>127677963</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>70.15492804999992</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>1372873</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>0.9457156999999998</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>7095255</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>13.62557925</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>32230252</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>18.26330005</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>13717170</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>7.847028049999998</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>14513746</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>8.859738050000006</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>30932694</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>18.30301069999999</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
         <v>4622790</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D60" s="3" t="n">
         <v>3.945586</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>427250</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>0.26789165</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr"/>
-      <c r="C38" s="5" t="n">
-        <v>863227233</v>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>605.8621873500003</v>
+      <c r="B62" s="4" t="inlineStr"/>
+      <c r="C62" s="5" t="n">
+        <v>2046658565</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>1426.238528</v>
       </c>
     </row>
   </sheetData>
@@ -1160,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1230,19 +1662,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>74476318</v>
+        <v>71591259</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>50.24984399999998</v>
+        <v>49.77146375000005</v>
       </c>
     </row>
     <row r="5">
@@ -1253,56 +1685,56 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>133765658</v>
+        <v>74476318</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>71.14932844999997</v>
+        <v>50.24984399999998</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>72187275</v>
+        <v>133765658</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>56.2498701</v>
+        <v>71.14932844999997</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>400375811</v>
+        <v>60816130</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>310.6193846500001</v>
+        <v>37.90077624999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1311,16 +1743,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>39476920</v>
+        <v>72187275</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>26.21059919999999</v>
+        <v>56.2498701</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1329,78 +1761,186 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7985488</v>
+        <v>400375811</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7.126000650000001</v>
+        <v>310.6193846500001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>93604273</v>
+        <v>91981189</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>48.35612305000001</v>
+        <v>67.75321470000004</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>34274081</v>
+        <v>39476920</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>29.42951395000001</v>
+        <v>26.21059919999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>7985488</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>7.126000650000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>641290060</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>483.1465527999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>93604273</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>48.35612305000001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>34274081</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>29.42951395000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>317325444</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>181.5364415</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RISKAZ-66573709-163a2507</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
         <v>4622790</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D17" s="3" t="n">
         <v>3.945586</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>427250</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.26789165</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="5" t="n">
-        <v>863227233</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>605.8621873500001</v>
+      <c r="B19" s="4" t="inlineStr"/>
+      <c r="C19" s="5" t="n">
+        <v>2046658565</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>1426.238528</v>
       </c>
     </row>
   </sheetData>
@@ -1414,7 +1954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1484,19 +2024,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>137703983</v>
+        <v>224388578</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>78.51230825</v>
+        <v>155.4254547000001</v>
       </c>
     </row>
     <row r="5">
@@ -1507,28 +2047,64 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
+        <v>137703983</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>78.51230825</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>42259569</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D6" s="3" t="n">
         <v>36.55551460000001</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tylers-PC-a0bfcb54</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>959042754</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>664.9508859499998</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
-      <c r="C6" s="5" t="n">
-        <v>863227233</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>605.8621873500002</v>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="5" t="n">
+        <v>2046658565</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1426.238528</v>
       </c>
     </row>
   </sheetData>
@@ -1542,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1583,27 +2159,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>1183431332</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>820.3763406499999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>578309299</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>419.4814096000002</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="n">
+        <v>419.4814096000001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>863227233</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>605.8621873500001</v>
+      <c r="B5" s="5" t="n">
+        <v>2046658565</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>1426.238528</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with revised data structure and metrics
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -643,10 +643,10 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>22622711</v>
+        <v>742219</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>13.7266725</v>
+        <v>0.4307016</v>
       </c>
     </row>
     <row r="11">
@@ -1568,17 +1568,269 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>8802350</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>4.531618</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>120920</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>0.45105125</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>5019</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>0.010495</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>7772265</v>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>8.370092649999998</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>2362</v>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>0.004116</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>20462565</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>10.7813003</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>197010264</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>90.56275129999975</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2025-12-23</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>18849663</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>11.9100709</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>114511667</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>53.65742795000001</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>142392344</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>81.10575265000014</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>37755362</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>34.68547765000002</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>54842226</v>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>49.12666164999995</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>46853881</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>42.37681665000003</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>28710781</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>20.92998685000001</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr"/>
-      <c r="C62" s="5" t="n">
-        <v>2046658565</v>
-      </c>
-      <c r="D62" s="6" t="n">
-        <v>1426.238528</v>
+      <c r="B76" s="4" t="inlineStr"/>
+      <c r="C76" s="5" t="n">
+        <v>2702869742</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>1821.4461759</v>
       </c>
     </row>
   </sheetData>
@@ -1592,7 +1844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1707,10 +1959,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>133765658</v>
+        <v>5561396</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>71.14932844999997</v>
+        <v>3.065023</v>
       </c>
     </row>
     <row r="7">
@@ -1930,17 +2182,89 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>37165481</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>24.1486732</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>330371594</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>156.1302501499998</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>234989932</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>164.9178919500001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>75564662</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>63.30680350000004</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="5" t="n">
-        <v>2046658565</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>1426.238528</v>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="5" t="n">
+        <v>2596545972</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>1766.65784135</v>
       </c>
     </row>
   </sheetData>
@@ -1954,7 +2278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2015,10 +2339,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>536049730</v>
+        <v>405937207</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>382.9258950000001</v>
+        <v>313.6844076500001</v>
       </c>
     </row>
     <row r="4">
@@ -2069,10 +2393,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>42259569</v>
+        <v>644786576</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.55551460000001</v>
+        <v>381.7523298999999</v>
       </c>
     </row>
     <row r="7">
@@ -2094,17 +2418,35 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>75637579</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>63.34610550000004</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="n">
-        <v>2046658565</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>1426.238528</v>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="5" t="n">
+        <v>2594710628</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1765.53996145</v>
       </c>
     </row>
   </sheetData>
@@ -2166,7 +2508,7 @@
         <v>1183431332</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>820.3763406499999</v>
+        <v>820.37634065</v>
       </c>
     </row>
     <row r="4">
@@ -2176,10 +2518,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>578309299</v>
+        <v>1234520476</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>419.4814096000001</v>
+        <v>814.6890575000001</v>
       </c>
     </row>
     <row r="5">
@@ -2189,10 +2531,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2046658565</v>
+        <v>2702869742</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>1426.238528</v>
+        <v>1821.4461759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with new data modifications
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1291,10 +1291,10 @@
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>26491616</v>
+        <v>22094757</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>11.8556978</v>
+        <v>9.632965449999997</v>
       </c>
     </row>
     <row r="47">
@@ -1624,25 +1624,25 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>7772265</v>
+        <v>223355</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>8.370092649999998</v>
+        <v>0.2059309</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1651,16 +1651,16 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>2362</v>
+        <v>7772265</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0.004116</v>
+        <v>8.370092649999998</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1669,16 +1669,16 @@
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>20462565</v>
+        <v>2362</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>10.7813003</v>
+        <v>0.004116</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1687,16 +1687,16 @@
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>197010264</v>
+        <v>20462565</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>90.56275129999975</v>
+        <v>10.7813003</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1705,16 +1705,16 @@
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>18849663</v>
+        <v>197010264</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>11.9100709</v>
+        <v>90.56275129999975</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1723,16 +1723,16 @@
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>114511667</v>
+        <v>18849663</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>53.65742795000001</v>
+        <v>11.9100709</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1741,16 +1741,16 @@
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>142392344</v>
+        <v>114511667</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>81.10575265000014</v>
+        <v>53.65742795000001</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1759,16 +1759,16 @@
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>37755362</v>
+        <v>142392344</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>34.68547765000002</v>
+        <v>81.10575265000014</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1777,16 +1777,16 @@
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>54842226</v>
+        <v>37755362</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>49.12666164999995</v>
+        <v>34.68547765000002</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1795,42 +1795,114 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>46853881</v>
+        <v>54842226</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>42.37681665000003</v>
+        <v>49.12666164999995</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>15956650</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>13.27670700000001</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>46853881</v>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>42.37681665000003</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>515719</v>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>0.5913671999999999</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>2026-01-08</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="n">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
         <v>28710781</v>
       </c>
-      <c r="D75" s="3" t="n">
+      <c r="D78" s="3" t="n">
         <v>20.92998685000001</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>56078109</v>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>35.38928375</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr"/>
-      <c r="C76" s="5" t="n">
-        <v>2702869742</v>
-      </c>
-      <c r="D76" s="6" t="n">
-        <v>1821.4461759</v>
+      <c r="B80" s="4" t="inlineStr"/>
+      <c r="C80" s="5" t="n">
+        <v>2771246716</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>1868.6867324</v>
       </c>
     </row>
   </sheetData>
@@ -1844,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2103,10 +2175,10 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>93604273</v>
+        <v>69215026</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>48.35612305000001</v>
+        <v>35.71718425</v>
       </c>
     </row>
     <row r="15">
@@ -2157,10 +2229,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>4622790</v>
+        <v>4846145</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>3.945586</v>
+        <v>4.151516900000001</v>
       </c>
     </row>
     <row r="18">
@@ -2254,17 +2326,35 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>72550478</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>49.25735795000001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="5" t="n">
-        <v>2596545972</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>1766.65784135</v>
+      <c r="B24" s="4" t="inlineStr"/>
+      <c r="C24" s="5" t="n">
+        <v>2644930558</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>1803.4821914</v>
       </c>
     </row>
   </sheetData>
@@ -2278,7 +2368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2375,10 +2465,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>137703983</v>
+        <v>74061171</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>78.51230825</v>
+        <v>39.86870115</v>
       </c>
     </row>
     <row r="6">
@@ -2436,17 +2526,35 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>72550478</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>49.25735795000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="5" t="n">
-        <v>2594710628</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>1765.53996145</v>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="5" t="n">
+        <v>2603618294</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1776.1537123</v>
       </c>
     </row>
   </sheetData>
@@ -2492,10 +2600,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>284917934</v>
+        <v>353294908</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>186.38077775</v>
+        <v>233.62133425</v>
       </c>
     </row>
     <row r="3">
@@ -2531,10 +2639,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2702869742</v>
+        <v>2771246716</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>1821.4461759</v>
+        <v>1868.6867324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with updated data modifications
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D80"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -670,19 +670,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>4554824</v>
+        <v>742219</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2.3443313</v>
+        <v>0.4307016</v>
       </c>
     </row>
     <row r="13">
@@ -693,236 +693,236 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>32445325</v>
+        <v>4554824</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>19.70108345</v>
+        <v>2.3443313</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>264353</v>
+        <v>32445325</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.2899901</v>
+        <v>19.70108345</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>25621364</v>
+        <v>4554824</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>16.1334694</v>
+        <v>2.3443313</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>24717634</v>
+        <v>264353</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>18.18267269999998</v>
+        <v>0.2899901</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>36196467</v>
+        <v>25621364</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>27.69193644999999</v>
+        <v>16.1334694</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>42282470</v>
+        <v>264353</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>34.37932540000001</v>
+        <v>0.2899901</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>134304301</v>
+        <v>24717634</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>111.3310283000001</v>
+        <v>18.18267269999998</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>5187171</v>
+        <v>36196467</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>3.687872</v>
+        <v>27.69193644999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>61197206</v>
+        <v>36196467</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>48.65078544999998</v>
+        <v>27.69193644999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>53296925</v>
+        <v>42282470</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>31.6186225</v>
+        <v>34.37932540000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>10092380</v>
+        <v>134304301</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>6.0643462</v>
+        <v>111.3310283000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>75311927</v>
+        <v>134304301</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>58.03115755000004</v>
+        <v>111.3310283000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>5756303</v>
+        <v>5187171</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>3.005845849999999</v>
+        <v>3.687872</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -931,88 +931,88 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>40068985</v>
+        <v>61197206</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>33.2958544</v>
+        <v>48.65078544999998</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-11-29</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>30795369</v>
+        <v>61197206</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>20.05914915000002</v>
+        <v>48.65078544999998</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>45337137</v>
+        <v>53296925</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>38.62387350000002</v>
+        <v>31.6186225</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>528925</v>
+        <v>10092380</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.38822715</v>
+        <v>6.0643462</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>13396201</v>
+        <v>53296925</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>13.78157245</v>
+        <v>31.6186225</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1021,16 +1021,16 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>350913</v>
+        <v>75311927</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.4064992500000001</v>
+        <v>58.03115755000004</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1039,34 +1039,34 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>55639860</v>
+        <v>5756303</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>44.61786230000001</v>
+        <v>3.005845849999999</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>24994881</v>
+        <v>75311927</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>16.63949649999999</v>
+        <v>58.03115755000004</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1075,16 +1075,16 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>251054</v>
+        <v>40068985</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.91434825</v>
+        <v>33.2958544</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1093,106 +1093,106 @@
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>41742778</v>
+        <v>30795369</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>31.88196614999998</v>
+        <v>20.05914915000002</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-29</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>6476688</v>
+        <v>40068985</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>4.3460157</v>
+        <v>33.2958544</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7383521</v>
+        <v>45337137</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>5.805153150000001</v>
+        <v>38.62387350000002</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>125222974</v>
+        <v>528925</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>109.86724235</v>
+        <v>0.38822715</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>7476426</v>
+        <v>13396201</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>4.83685985</v>
+        <v>13.78157245</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>129389519</v>
+        <v>350913</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>89.77331820000003</v>
+        <v>0.4064992500000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1201,34 +1201,34 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>182790445</v>
+        <v>55639860</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>131.8210713499999</v>
+        <v>44.61786230000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2025-12-07</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>93108283</v>
+        <v>350913</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>61.40351999999999</v>
+        <v>0.4064992500000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1237,16 +1237,16 @@
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>19992388</v>
+        <v>24994881</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>10.41620645</v>
+        <v>16.63949649999999</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1255,16 +1255,16 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>84554</v>
+        <v>251054</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.34924275</v>
+        <v>0.91434825</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1273,106 +1273,106 @@
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>28210903</v>
+        <v>41742778</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>14.03307105000002</v>
+        <v>31.88196614999998</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>22094757</v>
+        <v>251054</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>9.632965449999997</v>
+        <v>0.91434825</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>10194888</v>
+        <v>6476688</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>5.0491626</v>
+        <v>4.3460157</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>30829943</v>
+        <v>7383521</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>17.43594785000001</v>
+        <v>5.805153150000001</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>326063</v>
+        <v>125222974</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>0.50919775</v>
+        <v>109.86724235</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>74361574</v>
+        <v>7383521</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>47.88594100000003</v>
+        <v>5.805153150000001</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1381,34 +1381,34 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>14917453</v>
+        <v>7476426</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>7.702555249999997</v>
+        <v>4.83685985</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>12254463</v>
+        <v>129389519</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>6.085756150000001</v>
+        <v>89.77331820000003</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-06</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1417,70 +1417,70 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>127677963</v>
+        <v>182790445</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>70.15492804999992</v>
+        <v>131.8210713499999</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>1372873</v>
+        <v>93108283</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>0.9457156999999998</v>
+        <v>61.40351999999999</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>7095255</v>
+        <v>19992388</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>13.62557925</v>
+        <v>10.41620645</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>32230252</v>
+        <v>84554</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>18.26330005</v>
+        <v>0.34924275</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2025-12-13</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1489,88 +1489,88 @@
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>13717170</v>
+        <v>28210903</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>7.847028049999998</v>
+        <v>14.03307105000002</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>14513746</v>
+        <v>84554</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>8.859738050000006</v>
+        <v>0.34924275</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2025-12-14</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>30932694</v>
+        <v>22094757</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>18.30301069999999</v>
+        <v>9.632965449999997</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>4622790</v>
+        <v>10194888</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>3.945586</v>
+        <v>5.0491626</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>427250</v>
+        <v>30829943</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>0.26789165</v>
+        <v>17.43594785000001</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1579,52 +1579,52 @@
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>8802350</v>
+        <v>326063</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>4.531618</v>
+        <v>0.50919775</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2025-12-17</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>120920</v>
+        <v>74361574</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0.45105125</v>
+        <v>47.88594100000003</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>5019</v>
+        <v>326063</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0.010495</v>
+        <v>0.50919775</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1633,16 +1633,16 @@
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>223355</v>
+        <v>14917453</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0.2059309</v>
+        <v>7.702555249999997</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1651,70 +1651,70 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>7772265</v>
+        <v>12254463</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>8.370092649999998</v>
+        <v>6.085756150000001</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>2362</v>
+        <v>127677963</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.004116</v>
+        <v>70.15492804999992</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>20462565</v>
+        <v>12254463</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>10.7813003</v>
+        <v>6.085756150000001</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>197010264</v>
+        <v>1372873</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>90.56275129999975</v>
+        <v>0.9457156999999998</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1723,70 +1723,70 @@
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>18849663</v>
+        <v>7095255</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>11.9100709</v>
+        <v>13.62557925</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>114511667</v>
+        <v>32230252</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>53.65742795000001</v>
+        <v>18.26330005</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>142392344</v>
+        <v>7095255</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>81.10575265000014</v>
+        <v>13.62557925</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-13</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>37755362</v>
+        <v>13717170</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>34.68547765000002</v>
+        <v>7.847028049999998</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1795,52 +1795,52 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>54842226</v>
+        <v>14513746</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>49.12666164999995</v>
+        <v>8.859738050000006</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>15956650</v>
+        <v>30932694</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>13.27670700000001</v>
+        <v>18.30301069999999</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2025-12-14</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>46853881</v>
+        <v>14513746</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>42.37681665000003</v>
+        <v>8.859738050000006</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1849,60 +1849,762 @@
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>515719</v>
+        <v>4622790</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>0.5913671999999999</v>
+        <v>3.945586</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>28710781</v>
+        <v>427250</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>20.92998685000001</v>
+        <v>0.26789165</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>8802350</v>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>4.531618</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>8802350</v>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>4.531618</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>120920</v>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>0.45105125</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>120920</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>0.45105125</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>5019</v>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>0.010495</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>223355</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0.2059309</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>5019</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>0.010495</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>7772265</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>8.370092649999998</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>7772265</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>8.370092649999998</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>2362</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>0.004116</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>2362</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0.004116</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>20462565</v>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>10.7813003</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>20462565</v>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>10.7813003</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>197010264</v>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>90.56275129999975</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>197010264</v>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>90.56275129999975</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2025-12-23</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>18849663</v>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>11.9100709</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2025-12-23</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>18849663</v>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>11.9100709</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>114511667</v>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>53.65742795000001</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>114511667</v>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>53.65742795000001</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>142392344</v>
+      </c>
+      <c r="D98" s="3" t="n">
+        <v>81.10575265000014</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>142392344</v>
+      </c>
+      <c r="D99" s="3" t="n">
+        <v>81.10575265000014</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>37755362</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>34.68547765000002</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="n">
+        <v>37755362</v>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>34.68547765000002</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>54842226</v>
+      </c>
+      <c r="D102" s="3" t="n">
+        <v>49.12666164999995</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="n">
+        <v>54842226</v>
+      </c>
+      <c r="D103" s="3" t="n">
+        <v>49.12666164999995</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="n">
+        <v>15956650</v>
+      </c>
+      <c r="D104" s="3" t="n">
+        <v>13.27670700000001</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="n">
+        <v>46853881</v>
+      </c>
+      <c r="D105" s="3" t="n">
+        <v>42.37681665000003</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="n">
+        <v>515719</v>
+      </c>
+      <c r="D106" s="3" t="n">
+        <v>0.5913671999999999</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>46853881</v>
+      </c>
+      <c r="D107" s="3" t="n">
+        <v>42.37681665000003</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
           <t>2026-01-08</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="n">
+        <v>28710781</v>
+      </c>
+      <c r="D108" s="3" t="n">
+        <v>20.92998685000001</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
         <is>
           <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
-      <c r="C79" s="2" t="n">
+      <c r="C109" s="2" t="n">
         <v>56078109</v>
       </c>
-      <c r="D79" s="3" t="n">
+      <c r="D109" s="3" t="n">
         <v>35.38928375</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="n">
+        <v>59190150</v>
+      </c>
+      <c r="D110" s="3" t="n">
+        <v>39.9736833</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="n">
+        <v>144213601</v>
+      </c>
+      <c r="D111" s="3" t="n">
+        <v>82.48471645000001</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="n">
+        <v>55442609</v>
+      </c>
+      <c r="D112" s="3" t="n">
+        <v>37.75470719999999</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="n">
+        <v>97652340</v>
+      </c>
+      <c r="D113" s="3" t="n">
+        <v>70.39617440000008</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="n">
+        <v>14226394</v>
+      </c>
+      <c r="D114" s="3" t="n">
+        <v>9.202008749999994</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v>110009010</v>
+      </c>
+      <c r="D115" s="3" t="n">
+        <v>76.77922750000002</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v>56273136</v>
+      </c>
+      <c r="D116" s="3" t="n">
+        <v>47.21099149999994</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="n">
+        <v>41862215</v>
+      </c>
+      <c r="D117" s="3" t="n">
+        <v>29.23827280000001</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="n">
+        <v>661814</v>
+      </c>
+      <c r="D118" s="3" t="n">
+        <v>0.8503498999999999</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr"/>
-      <c r="C80" s="5" t="n">
-        <v>2771246716</v>
-      </c>
-      <c r="D80" s="6" t="n">
-        <v>1868.6867324</v>
+      <c r="B119" s="4" t="inlineStr"/>
+      <c r="C119" s="5" t="n">
+        <v>4448355649</v>
+      </c>
+      <c r="D119" s="6" t="n">
+        <v>3000.390418400002</v>
       </c>
     </row>
   </sheetData>
@@ -1916,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2058,19 +2760,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>72187275</v>
+        <v>5561396</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>56.2498701</v>
+        <v>3.065023</v>
       </c>
     </row>
     <row r="9">
@@ -2081,14 +2783,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>400375811</v>
+        <v>72187275</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>310.6193846500001</v>
+        <v>56.2498701</v>
       </c>
     </row>
     <row r="10">
@@ -2099,50 +2801,50 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>91981189</v>
+        <v>400375811</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>67.75321470000004</v>
+        <v>310.6193846500001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>39476920</v>
+        <v>91981189</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>26.21059919999999</v>
+        <v>67.75321470000004</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>7985488</v>
+        <v>400375811</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7.126000650000001</v>
+        <v>310.6193846500001</v>
       </c>
     </row>
     <row r="13">
@@ -2153,74 +2855,74 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>641290060</v>
+        <v>39476920</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>483.1465527999999</v>
+        <v>26.21059919999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>69215026</v>
+        <v>7985488</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>35.71718425</v>
+        <v>7.126000650000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>34274081</v>
+        <v>641290060</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>29.42951395000001</v>
+        <v>483.1465527999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>317325444</v>
+        <v>7985488</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>181.5364415</v>
+        <v>7.126000650000001</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2229,132 +2931,294 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>4846145</v>
+        <v>69215026</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>4.151516900000001</v>
+        <v>35.71718425</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>427250</v>
+        <v>34274081</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.26789165</v>
+        <v>29.42951395000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>37165481</v>
+        <v>317325444</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>24.1486732</v>
+        <v>181.5364415</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>330371594</v>
+        <v>34274081</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>156.1302501499998</v>
+        <v>29.42951395000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>234989932</v>
+        <v>4846145</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>164.9178919500001</v>
+        <v>4.151516900000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>75564662</v>
+        <v>427250</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>63.30680350000004</v>
+        <v>0.26789165</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>37165481</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>24.1486732</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>37165481</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>24.1486732</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>330371594</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>156.1302501499998</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>330371594</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>156.1302501499998</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>234989932</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>164.9178919500001</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>234989932</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>164.9178919500001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>75564662</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>63.30680350000004</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C30" s="2" t="n">
         <v>72550478</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D30" s="3" t="n">
         <v>49.25735795000001</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>403352581</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>272.9860980000001</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>223032569</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>163.2808504499999</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="5" t="n">
-        <v>2644930558</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>1803.4821914</v>
+      <c r="B33" s="4" t="inlineStr"/>
+      <c r="C33" s="5" t="n">
+        <v>4322039491</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>2935.185877399999</v>
       </c>
     </row>
   </sheetData>
@@ -2368,7 +3232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2456,19 +3320,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RISKAZ-66573709-163a2507</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>74061171</v>
+        <v>405937207</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>39.86870115</v>
+        <v>313.6844076500001</v>
       </c>
     </row>
     <row r="6">
@@ -2479,14 +3343,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>644786576</v>
+        <v>74061171</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>381.7523298999999</v>
+        <v>39.86870115</v>
       </c>
     </row>
     <row r="7">
@@ -2497,64 +3361,118 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tylers-PC-a0bfcb54</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>959042754</v>
+        <v>644786576</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>664.9508859499998</v>
+        <v>381.7523298999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>Tylers-PC-a0bfcb54</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>75637579</v>
+        <v>959042754</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>63.34610550000004</v>
+        <v>664.9508859499998</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>644786576</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>381.7523298999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>75637579</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>63.34610550000004</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C11" s="2" t="n">
         <v>72550478</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D11" s="3" t="n">
         <v>49.25735795000001</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>626385150</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>436.2669484500001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="5" t="n">
-        <v>2603618294</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>1776.1537123</v>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="5" t="n">
+        <v>4280727227</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>2907.8573983</v>
       </c>
     </row>
   </sheetData>
@@ -2568,7 +3486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2633,16 +3551,29 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1677108933</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1131.703686</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>2771246716</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>1868.6867324</v>
+      <c r="B6" s="5" t="n">
+        <v>4448355649</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>3000.3904184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with data modifications
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2731,24 +2731,96 @@
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>11873502</v>
+        <v>108562877</v>
       </c>
       <c r="D126" s="3" t="n">
-        <v>15.616441</v>
+        <v>79.70983509999976</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="4" t="inlineStr">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v>65801459</v>
+      </c>
+      <c r="D127" s="3" t="n">
+        <v>46.37876080000003</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="n">
+        <v>6261036</v>
+      </c>
+      <c r="D128" s="3" t="n">
+        <v>5.352366500000002</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="n">
+        <v>135757209</v>
+      </c>
+      <c r="D129" s="3" t="n">
+        <v>88.53619544999998</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="n">
+        <v>54050998</v>
+      </c>
+      <c r="D130" s="3" t="n">
+        <v>37.81899174999998</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B127" s="4" t="inlineStr"/>
-      <c r="C127" s="5" t="n">
-        <v>4875476799</v>
-      </c>
-      <c r="D127" s="6" t="n">
-        <v>3336.054103350002</v>
+      <c r="B131" s="4" t="inlineStr"/>
+      <c r="C131" s="5" t="n">
+        <v>5234036876</v>
+      </c>
+      <c r="D131" s="6" t="n">
+        <v>3578.233811950002</v>
       </c>
     </row>
   </sheetData>
@@ -3381,10 +3453,10 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>11873502</v>
+        <v>370613847</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>15.616441</v>
+        <v>257.8961340999998</v>
       </c>
     </row>
     <row r="35">
@@ -3395,10 +3467,10 @@
       </c>
       <c r="B35" s="4" t="inlineStr"/>
       <c r="C35" s="5" t="n">
-        <v>4744537851</v>
+        <v>5103278196</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>3266.90397635</v>
+        <v>3509.18366945</v>
       </c>
     </row>
   </sheetData>
@@ -3635,10 +3707,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1011666135</v>
+        <v>1370510284</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>738.6150959</v>
+        <v>980.9821927499997</v>
       </c>
     </row>
     <row r="13">
@@ -3649,10 +3721,10 @@
       </c>
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="5" t="n">
-        <v>4634098866</v>
+        <v>4992943015</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3203.902725</v>
+        <v>3446.26982185</v>
       </c>
     </row>
   </sheetData>
@@ -3737,10 +3809,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2062301613</v>
+        <v>2420861690</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1434.00742145</v>
+        <v>1676.187130049999</v>
       </c>
     </row>
     <row r="6">
@@ -3750,10 +3822,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4875476799</v>
+        <v>5234036876</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3336.05410335</v>
+        <v>3578.23381195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with changes
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2803,24 +2803,96 @@
         </is>
       </c>
       <c r="C130" s="2" t="n">
-        <v>54050998</v>
+        <v>222792084</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>37.81899174999998</v>
+        <v>150.0448951499998</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="4" t="inlineStr">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="n">
+        <v>31192250</v>
+      </c>
+      <c r="D131" s="3" t="n">
+        <v>22.40136895</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="n">
+        <v>7790210</v>
+      </c>
+      <c r="D132" s="3" t="n">
+        <v>6.031818</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="n">
+        <v>17492201</v>
+      </c>
+      <c r="D133" s="3" t="n">
+        <v>11.9030614</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="n">
+        <v>93448873</v>
+      </c>
+      <c r="D134" s="3" t="n">
+        <v>54.03199825000004</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B131" s="4" t="inlineStr"/>
-      <c r="C131" s="5" t="n">
-        <v>5234036876</v>
-      </c>
-      <c r="D131" s="6" t="n">
-        <v>3578.233811950002</v>
+      <c r="B135" s="4" t="inlineStr"/>
+      <c r="C135" s="5" t="n">
+        <v>5552701496</v>
+      </c>
+      <c r="D135" s="6" t="n">
+        <v>3784.827961950001</v>
       </c>
     </row>
   </sheetData>
@@ -2834,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3453,24 +3525,42 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>370613847</v>
+        <v>578157125</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>257.8961340999998</v>
+        <v>398.4552399499996</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>111041925</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>65.98770315000004</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="5" t="n">
-        <v>5103278196</v>
-      </c>
-      <c r="D35" s="6" t="n">
-        <v>3509.18366945</v>
+      <c r="B36" s="4" t="inlineStr"/>
+      <c r="C36" s="5" t="n">
+        <v>5421863399</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>3715.730478449999</v>
       </c>
     </row>
   </sheetData>
@@ -3707,10 +3797,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1370510284</v>
+        <v>1688903378</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>980.9821927499997</v>
+        <v>1187.397185999999</v>
       </c>
     </row>
     <row r="13">
@@ -3721,10 +3811,10 @@
       </c>
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="5" t="n">
-        <v>4992943015</v>
+        <v>5311336109</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3446.26982185</v>
+        <v>3652.684815099999</v>
       </c>
     </row>
   </sheetData>
@@ -3809,10 +3899,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2420861690</v>
+        <v>2739526310</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1676.187130049999</v>
+        <v>1882.781280049999</v>
       </c>
     </row>
     <row r="6">
@@ -3822,10 +3912,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>5234036876</v>
+        <v>5552701496</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3578.23381195</v>
+        <v>3784.82796195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with modifications
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2875,24 +2875,60 @@
         </is>
       </c>
       <c r="C134" s="2" t="n">
-        <v>138117215</v>
+        <v>191061123</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>80.05171874999996</v>
+        <v>110.4232795500001</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="4" t="inlineStr">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="n">
+        <v>12986670</v>
+      </c>
+      <c r="D135" s="3" t="n">
+        <v>10.14750310000001</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="n">
+        <v>58614253</v>
+      </c>
+      <c r="D136" s="3" t="n">
+        <v>33.87104950000001</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B135" s="4" t="inlineStr"/>
-      <c r="C135" s="5" t="n">
-        <v>5597369838</v>
-      </c>
-      <c r="D135" s="6" t="n">
-        <v>3810.847682450001</v>
+      <c r="B137" s="4" t="inlineStr"/>
+      <c r="C137" s="5" t="n">
+        <v>5721914669</v>
+      </c>
+      <c r="D137" s="6" t="n">
+        <v>3885.237795850001</v>
       </c>
     </row>
   </sheetData>
@@ -3543,10 +3579,10 @@
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>155714361</v>
+        <v>280289720</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>92.01915689999996</v>
+        <v>166.4282275500001</v>
       </c>
     </row>
     <row r="36">
@@ -3557,10 +3593,10 @@
       </c>
       <c r="B36" s="4" t="inlineStr"/>
       <c r="C36" s="5" t="n">
-        <v>5466535835</v>
+        <v>5591111194</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>3741.761932199999</v>
+        <v>3816.171002849999</v>
       </c>
     </row>
   </sheetData>
@@ -3797,10 +3833,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1733681087</v>
+        <v>1858151173</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1213.48322975</v>
+        <v>1287.837710399999</v>
       </c>
     </row>
     <row r="13">
@@ -3811,10 +3847,10 @@
       </c>
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="5" t="n">
-        <v>5356113818</v>
+        <v>5480583904</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3678.77085885</v>
+        <v>3753.125339499999</v>
       </c>
     </row>
   </sheetData>
@@ -3899,10 +3935,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2784194652</v>
+        <v>2908739483</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1908.801000549999</v>
+        <v>1983.191113949999</v>
       </c>
     </row>
     <row r="6">
@@ -3912,10 +3948,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>5597369838</v>
+        <v>5721914669</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3810.847682449999</v>
+        <v>3885.23779585</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add .breadcrumbs.json file with initial structure
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D179"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3674,17 +3674,35 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="4" t="inlineStr">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Mac.lan-dbb5a60e</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="n">
+        <v>607455</v>
+      </c>
+      <c r="D179" s="3" t="n">
+        <v>0.43856975</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B179" s="4" t="inlineStr"/>
-      <c r="C179" s="5" t="n">
-        <v>8546832123</v>
-      </c>
-      <c r="D179" s="6" t="n">
-        <v>5892.578990850005</v>
+      <c r="B180" s="4" t="inlineStr"/>
+      <c r="C180" s="5" t="n">
+        <v>8547439578</v>
+      </c>
+      <c r="D180" s="6" t="n">
+        <v>5893.017560600005</v>
       </c>
     </row>
   </sheetData>
@@ -4515,10 +4533,10 @@
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>60877874</v>
+        <v>61485329</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46.82114130000004</v>
+        <v>47.25971105000004</v>
       </c>
     </row>
     <row r="46">
@@ -4529,10 +4547,10 @@
       </c>
       <c r="B46" s="4" t="inlineStr"/>
       <c r="C46" s="5" t="n">
-        <v>8183330332</v>
+        <v>8183937787</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>5707.58866875</v>
+        <v>5708.0272385</v>
       </c>
     </row>
   </sheetData>
@@ -4841,10 +4859,10 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>318283526</v>
+        <v>318890981</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>275.3313962499999</v>
+        <v>275.7699659999999</v>
       </c>
     </row>
     <row r="17">
@@ -4855,10 +4873,10 @@
       </c>
       <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="5" t="n">
-        <v>8030543473</v>
+        <v>8031150928</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>5607.987490799997</v>
+        <v>5608.426060549998</v>
       </c>
     </row>
   </sheetData>
@@ -4904,10 +4922,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>2556887596</v>
+        <v>2557495051</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1785.636666449999</v>
+        <v>1786.075236199999</v>
       </c>
     </row>
     <row r="3">
@@ -4969,10 +4987,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8546832123</v>
+        <v>8547439578</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>5892.578990849999</v>
+        <v>5893.017560599999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with new data
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machine Totals" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Daily" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Machine Totals" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3604,19 +3604,19 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-c4e297c3</t>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
         </is>
       </c>
       <c r="C175" s="2" t="n">
-        <v>4176546</v>
+        <v>75111</v>
       </c>
       <c r="D175" s="3" t="n">
-        <v>4.82668475</v>
+        <v>0.1229025</v>
       </c>
     </row>
     <row r="176">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Mac.lan-dbb5a60e</t>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
         </is>
       </c>
       <c r="C176" s="2" t="n">
@@ -3640,7 +3640,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -3649,60 +3649,222 @@
         </is>
       </c>
       <c r="C177" s="2" t="n">
-        <v>52903901</v>
+        <v>4176546</v>
       </c>
       <c r="D177" s="3" t="n">
-        <v>41.71930155000003</v>
+        <v>4.82668475</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Mac.lan-dbb5a60e</t>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
-        <v>7973973</v>
+        <v>175750093</v>
       </c>
       <c r="D178" s="3" t="n">
-        <v>5.10183975</v>
+        <v>99.86452054999997</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="n">
+        <v>89412827</v>
+      </c>
+      <c r="D179" s="3" t="n">
+        <v>58.31839669999993</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="n">
+        <v>119474424</v>
+      </c>
+      <c r="D180" s="3" t="n">
+        <v>76.56217229999987</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="n">
+        <v>141282945</v>
+      </c>
+      <c r="D181" s="3" t="n">
+        <v>95.11837634999998</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Mac.lan-dbb5a60e</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="n">
+        <v>52903901</v>
+      </c>
+      <c r="D182" s="3" t="n">
+        <v>41.71930155000003</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="n">
+        <v>278509973</v>
+      </c>
+      <c r="D183" s="3" t="n">
+        <v>192.7719502999993</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="n">
+        <v>205485410</v>
+      </c>
+      <c r="D184" s="3" t="n">
+        <v>128.1476708</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Mac.lan-dbb5a60e</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="n">
+        <v>7973973</v>
+      </c>
+      <c r="D185" s="3" t="n">
+        <v>5.10183975</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="n">
+        <v>129097351</v>
+      </c>
+      <c r="D186" s="3" t="n">
+        <v>82.47942709999988</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
           <t>2026-02-12</t>
         </is>
       </c>
-      <c r="B179" t="inlineStr">
+      <c r="B187" t="inlineStr">
         <is>
           <t>Mac.lan-dbb5a60e</t>
         </is>
       </c>
-      <c r="C179" s="2" t="n">
+      <c r="C187" s="2" t="n">
         <v>607455</v>
       </c>
-      <c r="D179" s="3" t="n">
+      <c r="D187" s="3" t="n">
         <v>0.43856975</v>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="4" t="inlineStr">
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="n">
+        <v>92791236</v>
+      </c>
+      <c r="D188" s="3" t="n">
+        <v>61.22118174999999</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B180" s="4" t="inlineStr"/>
-      <c r="C180" s="5" t="n">
-        <v>8547439578</v>
-      </c>
-      <c r="D180" s="6" t="n">
-        <v>5893.017560600005</v>
+      <c r="B189" s="4" t="inlineStr"/>
+      <c r="C189" s="5" t="n">
+        <v>9779318948</v>
+      </c>
+      <c r="D189" s="6" t="n">
+        <v>6687.624158950003</v>
       </c>
     </row>
   </sheetData>
@@ -3716,7 +3878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4524,33 +4686,69 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>525995400</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>329.9863683999997</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>2026-02-09</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Mac.lan-dbb5a60e</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C46" s="2" t="n">
         <v>61485329</v>
       </c>
-      <c r="D45" s="3" t="n">
+      <c r="D46" s="3" t="n">
         <v>47.25971105000004</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>705883970</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>464.6202299499992</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr"/>
-      <c r="C46" s="5" t="n">
-        <v>8183937787</v>
-      </c>
-      <c r="D46" s="6" t="n">
-        <v>5708.0272385</v>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="5" t="n">
+        <v>9415817157</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>6502.633836849998</v>
       </c>
     </row>
   </sheetData>
@@ -4564,7 +4762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4866,17 +5064,35 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1231879370</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>794.6065983499989</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="5" t="n">
-        <v>8031150928</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>5608.426060549998</v>
+      <c r="B18" s="4" t="inlineStr"/>
+      <c r="C18" s="5" t="n">
+        <v>9263030298</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>6403.032658899996</v>
       </c>
     </row>
   </sheetData>
@@ -4890,7 +5106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4957,40 +5173,53 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-ab71ee47</t>
+          <t>tylers-Mac-mini-10.lan-09ef2ada</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1234520476</v>
+        <v>1231879370</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>814.6890575000001</v>
+        <v>794.6065983499989</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tylers-MacBook-Air.local-c4e297c3</t>
+          <t>tylers-MacBook-Air.local-ab71ee47</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
+        <v>1234520476</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>814.6890575000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tylers-MacBook-Air.local-c4e297c3</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>3176769341</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C7" s="3" t="n">
         <v>2204.8956425</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>8547439578</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>5893.017560599999</v>
+      <c r="B8" s="5" t="n">
+        <v>9779318948</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>6687.624158949998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove unused configuration files and update usage_tracker.xlsx
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D224"/>
+  <dimension ref="A1:D247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3883,10 +3883,10 @@
         </is>
       </c>
       <c r="C190" s="2" t="n">
-        <v>175750093</v>
+        <v>3433187</v>
       </c>
       <c r="D190" s="3" t="n">
-        <v>99.86452054999997</v>
+        <v>2.0279453</v>
       </c>
     </row>
     <row r="191">
@@ -3937,10 +3937,10 @@
         </is>
       </c>
       <c r="C193" s="2" t="n">
-        <v>89412827</v>
+        <v>10967620</v>
       </c>
       <c r="D193" s="3" t="n">
-        <v>58.31839669999993</v>
+        <v>7.964795699999998</v>
       </c>
     </row>
     <row r="194">
@@ -3973,10 +3973,10 @@
         </is>
       </c>
       <c r="C195" s="2" t="n">
-        <v>119474424</v>
+        <v>8467699</v>
       </c>
       <c r="D195" s="3" t="n">
-        <v>76.56217229999987</v>
+        <v>5.662390049999998</v>
       </c>
     </row>
     <row r="196">
@@ -4009,10 +4009,10 @@
         </is>
       </c>
       <c r="C197" s="2" t="n">
-        <v>141282945</v>
+        <v>15649426</v>
       </c>
       <c r="D197" s="3" t="n">
-        <v>95.11837634999998</v>
+        <v>10.63269685</v>
       </c>
     </row>
     <row r="198">
@@ -4063,10 +4063,10 @@
         </is>
       </c>
       <c r="C200" s="2" t="n">
-        <v>278509973</v>
+        <v>141222741</v>
       </c>
       <c r="D200" s="3" t="n">
-        <v>192.7719502999993</v>
+        <v>91.70154065000014</v>
       </c>
     </row>
     <row r="201">
@@ -4099,10 +4099,10 @@
         </is>
       </c>
       <c r="C202" s="2" t="n">
-        <v>205485410</v>
+        <v>24399351</v>
       </c>
       <c r="D202" s="3" t="n">
-        <v>128.1476708</v>
+        <v>11.11900180000001</v>
       </c>
     </row>
     <row r="203">
@@ -4171,10 +4171,10 @@
         </is>
       </c>
       <c r="C206" s="2" t="n">
-        <v>129097351</v>
+        <v>21477360</v>
       </c>
       <c r="D206" s="3" t="n">
-        <v>82.47942709999988</v>
+        <v>12.37667285</v>
       </c>
     </row>
     <row r="207">
@@ -4243,10 +4243,10 @@
         </is>
       </c>
       <c r="C210" s="2" t="n">
-        <v>92791236</v>
+        <v>19518241</v>
       </c>
       <c r="D210" s="3" t="n">
-        <v>61.22118174999999</v>
+        <v>14.22901225000001</v>
       </c>
     </row>
     <row r="211">
@@ -4261,10 +4261,10 @@
         </is>
       </c>
       <c r="C211" s="2" t="n">
-        <v>160938583</v>
+        <v>44477831</v>
       </c>
       <c r="D211" s="3" t="n">
-        <v>110.5201702499998</v>
+        <v>26.24059799999999</v>
       </c>
     </row>
     <row r="212">
@@ -4279,10 +4279,10 @@
         </is>
       </c>
       <c r="C212" s="2" t="n">
-        <v>346688764</v>
+        <v>146818569</v>
       </c>
       <c r="D212" s="3" t="n">
-        <v>220.0138839499999</v>
+        <v>99.50533869999997</v>
       </c>
     </row>
     <row r="213">
@@ -4315,10 +4315,10 @@
         </is>
       </c>
       <c r="C214" s="2" t="n">
-        <v>84150122</v>
+        <v>5702830</v>
       </c>
       <c r="D214" s="3" t="n">
-        <v>55.29194370000009</v>
+        <v>4.375258700000001</v>
       </c>
     </row>
     <row r="215">
@@ -4333,10 +4333,10 @@
         </is>
       </c>
       <c r="C215" s="2" t="n">
-        <v>45288788</v>
+        <v>4990024</v>
       </c>
       <c r="D215" s="3" t="n">
-        <v>47.22257775000001</v>
+        <v>4.048521749999999</v>
       </c>
     </row>
     <row r="216">
@@ -4484,17 +4484,431 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="4" t="inlineStr">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="n">
+        <v>215163169</v>
+      </c>
+      <c r="D224" s="3" t="n">
+        <v>147.1839522499998</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="n">
+        <v>432850555</v>
+      </c>
+      <c r="D225" s="3" t="n">
+        <v>267.1754671500002</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="n">
+        <v>365235184</v>
+      </c>
+      <c r="D226" s="3" t="n">
+        <v>225.5522911500005</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="n">
+        <v>352423151</v>
+      </c>
+      <c r="D227" s="3" t="n">
+        <v>215.5466881999997</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="n">
+        <v>452317726</v>
+      </c>
+      <c r="D228" s="3" t="n">
+        <v>272.4973686000004</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="n">
+        <v>182612831</v>
+      </c>
+      <c r="D229" s="3" t="n">
+        <v>114.1695863000002</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="n">
+        <v>24062714</v>
+      </c>
+      <c r="D230" s="3" t="n">
+        <v>16.47748660000001</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="n">
+        <v>258592616</v>
+      </c>
+      <c r="D231" s="3" t="n">
+        <v>164.7672837499995</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="n">
+        <v>117225840</v>
+      </c>
+      <c r="D232" s="3" t="n">
+        <v>72.61162089999992</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="n">
+        <v>229961706</v>
+      </c>
+      <c r="D233" s="3" t="n">
+        <v>147.1799392499997</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="n">
+        <v>149672659</v>
+      </c>
+      <c r="D234" s="3" t="n">
+        <v>92.61565039999995</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="n">
+        <v>172481053</v>
+      </c>
+      <c r="D235" s="3" t="n">
+        <v>105.7200134999999</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="n">
+        <v>248660819</v>
+      </c>
+      <c r="D236" s="3" t="n">
+        <v>161.5157197</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="n">
+        <v>142960439</v>
+      </c>
+      <c r="D237" s="3" t="n">
+        <v>83.47115404999988</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="n">
+        <v>290300157</v>
+      </c>
+      <c r="D238" s="3" t="n">
+        <v>185.5870636500007</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="n">
+        <v>62870675</v>
+      </c>
+      <c r="D239" s="3" t="n">
+        <v>37.33927440000003</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="n">
+        <v>186347353</v>
+      </c>
+      <c r="D240" s="3" t="n">
+        <v>123.5888548999999</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="n">
+        <v>482385077</v>
+      </c>
+      <c r="D241" s="3" t="n">
+        <v>315.5251320499994</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="n">
+        <v>3191943</v>
+      </c>
+      <c r="D242" s="3" t="n">
+        <v>2.2486859</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="n">
+        <v>382332777</v>
+      </c>
+      <c r="D243" s="3" t="n">
+        <v>286.28041865</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="n">
+        <v>280689768</v>
+      </c>
+      <c r="D244" s="3" t="n">
+        <v>167.9958539499999</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="n">
+        <v>226524840</v>
+      </c>
+      <c r="D245" s="3" t="n">
+        <v>157.9753783</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="n">
+        <v>32177340</v>
+      </c>
+      <c r="D246" s="3" t="n">
+        <v>21.85533164999999</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B224" s="4" t="inlineStr"/>
-      <c r="C224" s="5" t="n">
-        <v>14609591326</v>
-      </c>
-      <c r="D224" s="6" t="n">
-        <v>9870.055544500001</v>
+      <c r="B247" s="4" t="inlineStr"/>
+      <c r="C247" s="5" t="n">
+        <v>18478886081</v>
+      </c>
+      <c r="D247" s="6" t="n">
+        <v>12317.28726085</v>
       </c>
     </row>
   </sheetData>
@@ -4508,7 +4922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5397,10 +5811,10 @@
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>525995400</v>
+        <v>38517932</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>329.9863683999997</v>
+        <v>26.2878279</v>
       </c>
     </row>
     <row r="50">
@@ -5469,10 +5883,10 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>1214289321</v>
+        <v>397914093</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>796.2403738999989</v>
+        <v>255.1721642500001</v>
       </c>
     </row>
     <row r="54">
@@ -5487,10 +5901,10 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>1507176466</v>
+        <v>1388430410</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>1082.741905199999</v>
+        <v>988.6511641999991</v>
       </c>
     </row>
     <row r="55">
@@ -5505,24 +5919,78 @@
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>1273144165</v>
+        <v>2638816224</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>761.3091272499989</v>
+        <v>1616.767525999999</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>1414446092</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>880.3189357999996</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>1586005573</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>1012.74721225</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>924916668</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>636.3556684499999</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr"/>
-      <c r="C56" s="5" t="n">
-        <v>14246089535</v>
-      </c>
-      <c r="D56" s="6" t="n">
-        <v>9685.065222399995</v>
+      <c r="B59" s="4" t="inlineStr"/>
+      <c r="C59" s="5" t="n">
+        <v>18114531175</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>12131.0879465</v>
       </c>
     </row>
   </sheetData>
@@ -5536,7 +6004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5885,24 +6353,42 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>4520605352</v>
+        <v>4111255508</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2970.277774749997</v>
+        <v>2671.331994149999</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>4277791484</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2744.968504699999</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr"/>
-      <c r="C20" s="5" t="n">
-        <v>14093302676</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>9585.464044449993</v>
+      <c r="B21" s="4" t="inlineStr"/>
+      <c r="C21" s="5" t="n">
+        <v>17961744316</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>12031.48676855</v>
       </c>
     </row>
   </sheetData>
@@ -6000,10 +6486,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4520605352</v>
+        <v>8389900107</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2970.277774749997</v>
+        <v>5417.509491099997</v>
       </c>
     </row>
     <row r="7">
@@ -6039,10 +6525,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>14609591326</v>
+        <v>18478886081</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>9870.055544499994</v>
+        <v>12317.28726084999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update usage_tracker.xlsx with revised data
</commit_message>
<xml_diff>
--- a/usage_tracker.xlsx
+++ b/usage_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machine Totals" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Daily" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Machine Totals" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D247"/>
+  <dimension ref="A1:D266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2767,10 +2767,10 @@
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>2243461</v>
+        <v>36306</v>
       </c>
       <c r="D128" s="3" t="n">
-        <v>1.532817</v>
+        <v>0.1130765</v>
       </c>
     </row>
     <row r="129">
@@ -2821,10 +2821,10 @@
         </is>
       </c>
       <c r="C131" s="2" t="n">
-        <v>16421163</v>
+        <v>915022</v>
       </c>
       <c r="D131" s="3" t="n">
-        <v>9.799548799999998</v>
+        <v>0.17475955</v>
       </c>
     </row>
     <row r="132">
@@ -2875,10 +2875,10 @@
         </is>
       </c>
       <c r="C134" s="2" t="n">
-        <v>18226055</v>
+        <v>1847812</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>17.50515954999999</v>
+        <v>0.2638230499999999</v>
       </c>
     </row>
     <row r="135">
@@ -2929,10 +2929,10 @@
         </is>
       </c>
       <c r="C137" s="2" t="n">
-        <v>41368313</v>
+        <v>1441698</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>35.98953820000004</v>
+        <v>1.2339702</v>
       </c>
     </row>
     <row r="138">
@@ -3109,10 +3109,10 @@
         </is>
       </c>
       <c r="C147" s="2" t="n">
-        <v>66080036</v>
+        <v>3020717</v>
       </c>
       <c r="D147" s="3" t="n">
-        <v>43.91275375000006</v>
+        <v>1.13627925</v>
       </c>
     </row>
     <row r="148">
@@ -3163,10 +3163,10 @@
         </is>
       </c>
       <c r="C150" s="2" t="n">
-        <v>10057463</v>
+        <v>2232464</v>
       </c>
       <c r="D150" s="3" t="n">
-        <v>7.677724099999999</v>
+        <v>0.4173436000000001</v>
       </c>
     </row>
     <row r="151">
@@ -3217,10 +3217,10 @@
         </is>
       </c>
       <c r="C153" s="2" t="n">
-        <v>1064164</v>
+        <v>749164</v>
       </c>
       <c r="D153" s="3" t="n">
-        <v>0.43412185</v>
+        <v>0.1607161</v>
       </c>
     </row>
     <row r="154">
@@ -3379,10 +3379,10 @@
         </is>
       </c>
       <c r="C162" s="2" t="n">
-        <v>17621529</v>
+        <v>453209</v>
       </c>
       <c r="D162" s="3" t="n">
-        <v>11.3690995</v>
+        <v>0.10620225</v>
       </c>
     </row>
     <row r="163">
@@ -3433,10 +3433,10 @@
         </is>
       </c>
       <c r="C165" s="2" t="n">
-        <v>97975155</v>
+        <v>3163742</v>
       </c>
       <c r="D165" s="3" t="n">
-        <v>65.01552019999997</v>
+        <v>1.11092345</v>
       </c>
     </row>
     <row r="166">
@@ -3487,10 +3487,10 @@
         </is>
       </c>
       <c r="C168" s="2" t="n">
-        <v>44732002</v>
+        <v>1077371</v>
       </c>
       <c r="D168" s="3" t="n">
-        <v>27.22697715</v>
+        <v>0.58071565</v>
       </c>
     </row>
     <row r="169">
@@ -3595,10 +3595,10 @@
         </is>
       </c>
       <c r="C174" s="2" t="n">
-        <v>16051221</v>
+        <v>5063541</v>
       </c>
       <c r="D174" s="3" t="n">
-        <v>10.82180295</v>
+        <v>2.680412699999999</v>
       </c>
     </row>
     <row r="175">
@@ -3721,10 +3721,10 @@
         </is>
       </c>
       <c r="C181" s="2" t="n">
-        <v>9957716</v>
+        <v>4310795</v>
       </c>
       <c r="D181" s="3" t="n">
-        <v>6.353663550000001</v>
+        <v>2.788559550000001</v>
       </c>
     </row>
     <row r="182">
@@ -3865,10 +3865,10 @@
         </is>
       </c>
       <c r="C189" s="2" t="n">
-        <v>31731358</v>
+        <v>1339409</v>
       </c>
       <c r="D189" s="3" t="n">
-        <v>18.19639385000002</v>
+        <v>0.42794685</v>
       </c>
     </row>
     <row r="190">
@@ -4153,10 +4153,10 @@
         </is>
       </c>
       <c r="C205" s="2" t="n">
-        <v>9003383</v>
+        <v>997440</v>
       </c>
       <c r="D205" s="3" t="n">
-        <v>5.090825849999997</v>
+        <v>0.1623111</v>
       </c>
     </row>
     <row r="206">
@@ -4225,10 +4225,10 @@
         </is>
       </c>
       <c r="C209" s="2" t="n">
-        <v>7866711</v>
+        <v>4994368</v>
       </c>
       <c r="D209" s="3" t="n">
-        <v>5.454199150000003</v>
+        <v>2.464812650000002</v>
       </c>
     </row>
     <row r="210">
@@ -4270,25 +4270,25 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C212" s="2" t="n">
-        <v>146818569</v>
+        <v>18810081</v>
       </c>
       <c r="D212" s="3" t="n">
-        <v>99.50533869999997</v>
+        <v>15.0921388</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -4297,16 +4297,16 @@
         </is>
       </c>
       <c r="C213" s="2" t="n">
-        <v>778004</v>
+        <v>146818569</v>
       </c>
       <c r="D213" s="3" t="n">
-        <v>1.08608975</v>
+        <v>99.50533869999997</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -4315,16 +4315,16 @@
         </is>
       </c>
       <c r="C214" s="2" t="n">
-        <v>5702830</v>
+        <v>778004</v>
       </c>
       <c r="D214" s="3" t="n">
-        <v>4.375258700000001</v>
+        <v>1.08608975</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -4333,16 +4333,16 @@
         </is>
       </c>
       <c r="C215" s="2" t="n">
-        <v>4990024</v>
+        <v>5702830</v>
       </c>
       <c r="D215" s="3" t="n">
-        <v>4.048521749999999</v>
+        <v>4.375258700000001</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -4351,16 +4351,16 @@
         </is>
       </c>
       <c r="C216" s="2" t="n">
-        <v>5148631</v>
+        <v>4990024</v>
       </c>
       <c r="D216" s="3" t="n">
-        <v>6.794404250000001</v>
+        <v>4.048521749999999</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -4369,16 +4369,16 @@
         </is>
       </c>
       <c r="C217" s="2" t="n">
-        <v>320134778</v>
+        <v>5148631</v>
       </c>
       <c r="D217" s="3" t="n">
-        <v>275.9560833999994</v>
+        <v>6.794404250000001</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -4387,34 +4387,34 @@
         </is>
       </c>
       <c r="C218" s="2" t="n">
-        <v>363424603</v>
+        <v>320134778</v>
       </c>
       <c r="D218" s="3" t="n">
-        <v>253.9949239</v>
+        <v>275.9560833999994</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C219" s="2" t="n">
-        <v>385168542</v>
+        <v>2637058</v>
       </c>
       <c r="D219" s="3" t="n">
-        <v>251.1209313999997</v>
+        <v>3.997989</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -4423,34 +4423,34 @@
         </is>
       </c>
       <c r="C220" s="2" t="n">
-        <v>303861002</v>
+        <v>363424603</v>
       </c>
       <c r="D220" s="3" t="n">
-        <v>192.3610407999999</v>
+        <v>253.9949239</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
-        <v>507372539</v>
+        <v>3235860</v>
       </c>
       <c r="D221" s="3" t="n">
-        <v>275.6535568499997</v>
+        <v>2.379956</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -4459,16 +4459,16 @@
         </is>
       </c>
       <c r="C222" s="2" t="n">
-        <v>521534498</v>
+        <v>385168542</v>
       </c>
       <c r="D222" s="3" t="n">
-        <v>307.5905128499994</v>
+        <v>251.1209313999997</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -4477,16 +4477,16 @@
         </is>
       </c>
       <c r="C223" s="2" t="n">
-        <v>244237128</v>
+        <v>303861002</v>
       </c>
       <c r="D223" s="3" t="n">
-        <v>178.0650575499999</v>
+        <v>192.3610407999999</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -4495,34 +4495,34 @@
         </is>
       </c>
       <c r="C224" s="2" t="n">
-        <v>215163169</v>
+        <v>507372539</v>
       </c>
       <c r="D224" s="3" t="n">
-        <v>147.1839522499998</v>
+        <v>275.6535568499997</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C225" s="2" t="n">
-        <v>432850555</v>
+        <v>2308354</v>
       </c>
       <c r="D225" s="3" t="n">
-        <v>267.1754671500002</v>
+        <v>1.877557199999998</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -4531,16 +4531,16 @@
         </is>
       </c>
       <c r="C226" s="2" t="n">
-        <v>365235184</v>
+        <v>521534498</v>
       </c>
       <c r="D226" s="3" t="n">
-        <v>225.5522911500005</v>
+        <v>307.5905128499994</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -4549,34 +4549,34 @@
         </is>
       </c>
       <c r="C227" s="2" t="n">
-        <v>352423151</v>
+        <v>244237128</v>
       </c>
       <c r="D227" s="3" t="n">
-        <v>215.5466881999997</v>
+        <v>178.0650575499999</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
-        <v>452317726</v>
+        <v>4307138</v>
       </c>
       <c r="D228" s="3" t="n">
-        <v>272.4973686000004</v>
+        <v>4.1447897</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -4585,16 +4585,16 @@
         </is>
       </c>
       <c r="C229" s="2" t="n">
-        <v>182612831</v>
+        <v>215163169</v>
       </c>
       <c r="D229" s="3" t="n">
-        <v>114.1695863000002</v>
+        <v>147.1839522499998</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -4603,34 +4603,34 @@
         </is>
       </c>
       <c r="C230" s="2" t="n">
-        <v>24062714</v>
+        <v>432850555</v>
       </c>
       <c r="D230" s="3" t="n">
-        <v>16.47748660000001</v>
+        <v>267.1754671500002</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C231" s="2" t="n">
-        <v>258592616</v>
+        <v>260226</v>
       </c>
       <c r="D231" s="3" t="n">
-        <v>164.7672837499995</v>
+        <v>0.1215106</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -4639,16 +4639,16 @@
         </is>
       </c>
       <c r="C232" s="2" t="n">
-        <v>117225840</v>
+        <v>365235184</v>
       </c>
       <c r="D232" s="3" t="n">
-        <v>72.61162089999992</v>
+        <v>225.5522911500005</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -4657,16 +4657,16 @@
         </is>
       </c>
       <c r="C233" s="2" t="n">
-        <v>229961706</v>
+        <v>352423151</v>
       </c>
       <c r="D233" s="3" t="n">
-        <v>147.1799392499997</v>
+        <v>215.5466881999997</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -4675,34 +4675,34 @@
         </is>
       </c>
       <c r="C234" s="2" t="n">
-        <v>149672659</v>
+        <v>452317726</v>
       </c>
       <c r="D234" s="3" t="n">
-        <v>92.61565039999995</v>
+        <v>272.4973686000004</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C235" s="2" t="n">
-        <v>172481053</v>
+        <v>57967225</v>
       </c>
       <c r="D235" s="3" t="n">
-        <v>105.7200134999999</v>
+        <v>36.33208630000001</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -4711,34 +4711,34 @@
         </is>
       </c>
       <c r="C236" s="2" t="n">
-        <v>248660819</v>
+        <v>182612831</v>
       </c>
       <c r="D236" s="3" t="n">
-        <v>161.5157197</v>
+        <v>114.1695863000002</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
-        <v>142960439</v>
+        <v>6212393</v>
       </c>
       <c r="D237" s="3" t="n">
-        <v>83.47115404999988</v>
+        <v>4.530312249999998</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -4747,34 +4747,34 @@
         </is>
       </c>
       <c r="C238" s="2" t="n">
-        <v>290300157</v>
+        <v>24062714</v>
       </c>
       <c r="D238" s="3" t="n">
-        <v>185.5870636500007</v>
+        <v>16.47748660000001</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C239" s="2" t="n">
-        <v>62870675</v>
+        <v>78344193</v>
       </c>
       <c r="D239" s="3" t="n">
-        <v>37.33927440000003</v>
+        <v>27.76409370000001</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -4783,34 +4783,34 @@
         </is>
       </c>
       <c r="C240" s="2" t="n">
-        <v>186347353</v>
+        <v>258592616</v>
       </c>
       <c r="D240" s="3" t="n">
-        <v>123.5888548999999</v>
+        <v>164.7672837499995</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C241" s="2" t="n">
-        <v>482385077</v>
+        <v>1280372</v>
       </c>
       <c r="D241" s="3" t="n">
-        <v>315.5251320499994</v>
+        <v>1.40290025</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -4819,16 +4819,16 @@
         </is>
       </c>
       <c r="C242" s="2" t="n">
-        <v>3191943</v>
+        <v>117225840</v>
       </c>
       <c r="D242" s="3" t="n">
-        <v>2.2486859</v>
+        <v>72.61162089999992</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -4837,16 +4837,16 @@
         </is>
       </c>
       <c r="C243" s="2" t="n">
-        <v>382332777</v>
+        <v>229961706</v>
       </c>
       <c r="D243" s="3" t="n">
-        <v>286.28041865</v>
+        <v>147.1799392499997</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -4855,16 +4855,16 @@
         </is>
       </c>
       <c r="C244" s="2" t="n">
-        <v>280689768</v>
+        <v>149672659</v>
       </c>
       <c r="D244" s="3" t="n">
-        <v>167.9958539499999</v>
+        <v>92.61565039999995</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -4873,42 +4873,384 @@
         </is>
       </c>
       <c r="C245" s="2" t="n">
-        <v>226524840</v>
+        <v>172481053</v>
       </c>
       <c r="D245" s="3" t="n">
-        <v>157.9753783</v>
+        <v>105.7200134999999</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="n">
+        <v>190447</v>
+      </c>
+      <c r="D246" s="3" t="n">
+        <v>0.26261195</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="n">
+        <v>248660819</v>
+      </c>
+      <c r="D247" s="3" t="n">
+        <v>161.5157197</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="n">
+        <v>59656</v>
+      </c>
+      <c r="D248" s="3" t="n">
+        <v>0.12231625</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="n">
+        <v>142960439</v>
+      </c>
+      <c r="D249" s="3" t="n">
+        <v>83.47115404999988</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="n">
+        <v>4043016</v>
+      </c>
+      <c r="D250" s="3" t="n">
+        <v>1.86714025</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="n">
+        <v>290300157</v>
+      </c>
+      <c r="D251" s="3" t="n">
+        <v>185.5870636500007</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="n">
+        <v>62870675</v>
+      </c>
+      <c r="D252" s="3" t="n">
+        <v>37.33927440000003</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="n">
+        <v>39049740</v>
+      </c>
+      <c r="D253" s="3" t="n">
+        <v>21.9178715</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="n">
+        <v>186347353</v>
+      </c>
+      <c r="D254" s="3" t="n">
+        <v>123.5888548999999</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="n">
+        <v>482385077</v>
+      </c>
+      <c r="D255" s="3" t="n">
+        <v>315.5251320499994</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="n">
+        <v>3191943</v>
+      </c>
+      <c r="D256" s="3" t="n">
+        <v>2.2486859</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="n">
+        <v>93030274</v>
+      </c>
+      <c r="D257" s="3" t="n">
+        <v>67.87805850000002</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="n">
+        <v>382332777</v>
+      </c>
+      <c r="D258" s="3" t="n">
+        <v>286.28041865</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="n">
+        <v>82900501</v>
+      </c>
+      <c r="D259" s="3" t="n">
+        <v>71.06402649999997</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="n">
+        <v>280689768</v>
+      </c>
+      <c r="D260" s="3" t="n">
+        <v>167.9958539499999</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="n">
+        <v>37416303</v>
+      </c>
+      <c r="D261" s="3" t="n">
+        <v>34.73157025000001</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="n">
+        <v>226524840</v>
+      </c>
+      <c r="D262" s="3" t="n">
+        <v>157.9753783</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="n">
+        <v>430527037</v>
+      </c>
+      <c r="D263" s="3" t="n">
+        <v>328.3051104500001</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="B246" t="inlineStr">
+      <c r="B264" t="inlineStr">
         <is>
           <t>tylers-Mac-mini.lan-033751f7</t>
         </is>
       </c>
-      <c r="C246" s="2" t="n">
+      <c r="C264" s="2" t="n">
         <v>32177340</v>
       </c>
-      <c r="D246" s="3" t="n">
+      <c r="D264" s="3" t="n">
         <v>21.85533164999999</v>
       </c>
     </row>
-    <row r="247">
-      <c r="A247" s="4" t="inlineStr">
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="n">
+        <v>31202108</v>
+      </c>
+      <c r="D265" s="3" t="n">
+        <v>24.23376025</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B247" s="4" t="inlineStr"/>
-      <c r="C247" s="5" t="n">
-        <v>18478886081</v>
-      </c>
-      <c r="D247" s="6" t="n">
-        <v>12317.28726085</v>
+      <c r="B266" s="4" t="inlineStr"/>
+      <c r="C266" s="5" t="n">
+        <v>19013911391</v>
+      </c>
+      <c r="D266" s="6" t="n">
+        <v>12712.75476755</v>
       </c>
     </row>
   </sheetData>
@@ -4922,7 +5264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5523,10 +5865,10 @@
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>31074048</v>
+        <v>84565</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>25.97423655</v>
+        <v>0.1117787</v>
       </c>
     </row>
     <row r="34">
@@ -5595,10 +5937,10 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>78258992</v>
+        <v>4240838</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>64.82706355000003</v>
+        <v>1.7856293</v>
       </c>
     </row>
     <row r="38">
@@ -5667,10 +6009,10 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>77201663</v>
+        <v>6002345</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>52.02459970000006</v>
+        <v>1.71433895</v>
       </c>
     </row>
     <row r="42">
@@ -5721,10 +6063,10 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>177321404</v>
+        <v>9757863</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>115.1280848</v>
+        <v>4.478254049999999</v>
       </c>
     </row>
     <row r="45">
@@ -5793,10 +6135,10 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>43419773</v>
+        <v>5650204</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>26.27190865000002</v>
+        <v>3.216506400000001</v>
       </c>
     </row>
     <row r="49">
@@ -5865,10 +6207,10 @@
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>16870094</v>
+        <v>24801889</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>10.545025</v>
+        <v>17.71926255</v>
       </c>
     </row>
     <row r="53">
@@ -5910,25 +6252,25 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>2638816224</v>
+        <v>5872918</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>1616.767525999999</v>
+        <v>6.377945</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5937,60 +6279,150 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>1414446092</v>
+        <v>2638816224</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>880.3189357999996</v>
+        <v>1616.767525999999</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>tylers-Mac-mini.lan-033751f7</t>
+          <t>RISKAZ-66573709-163a2507</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>1586005573</v>
+        <v>6875718</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>1012.74721225</v>
+        <v>6.143857499999998</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>1414446092</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>880.3189357999996</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>143804183</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>70.02939250000001</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>tylers-Mac-mini.lan-033751f7</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>1586005573</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>1012.74721225</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>43342859</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>24.16993995</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>tylers-Mac-mini.lan-033751f7</t>
         </is>
       </c>
-      <c r="C58" s="2" t="n">
+      <c r="C62" s="2" t="n">
         <v>924916668</v>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="D62" s="3" t="n">
         <v>636.3556684499999</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>675076223</v>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>526.2125259500002</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr"/>
-      <c r="C59" s="5" t="n">
-        <v>18114531175</v>
-      </c>
-      <c r="D59" s="6" t="n">
-        <v>12131.0879465</v>
+      <c r="B64" s="4" t="inlineStr"/>
+      <c r="C64" s="5" t="n">
+        <v>18615894806</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>12498.2764591</v>
       </c>
     </row>
   </sheetData>
@@ -6004,7 +6436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6227,10 +6659,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>363856107</v>
+        <v>20085611</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>257.9539846000001</v>
+        <v>8.090000999999999</v>
       </c>
     </row>
     <row r="13">
@@ -6335,10 +6767,10 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>60289867</v>
+        <v>43200729</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>36.81693365000002</v>
+        <v>33.45757145</v>
       </c>
     </row>
     <row r="19">
@@ -6378,17 +6810,35 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RISKAZ-66573709-163a2507</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>862223265</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>620.4118584000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="5" t="n">
-        <v>17961744316</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>12031.48676855</v>
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="5" t="n">
+        <v>18463107947</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>12398.67528114999</v>
       </c>
     </row>
   </sheetData>
@@ -6447,10 +6897,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>704890404</v>
+        <v>1239915714</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>479.13489455</v>
+        <v>874.6024012500001</v>
       </c>
     </row>
     <row r="4">
@@ -6525,10 +6975,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>18478886081</v>
+        <v>19013911391</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>12317.28726084999</v>
+        <v>12712.75476755</v>
       </c>
     </row>
   </sheetData>

</xml_diff>